<commit_message>
QA+E2E: logo transparente, fix FAB del carrito, barra de pago amarilla, variantes de talla/color en ficha y mensaje, barrio opcional, sin placeholders, checkout fullscreen en movil; sync automatico de los 4 catalogos (cron 6h) con catalogo.js externo y Excel actualizados
</commit_message>
<xml_diff>
--- a/Jugueteria_Taiwan_Catalogo.xlsx
+++ b/Jugueteria_Taiwan_Catalogo.xlsx
@@ -82,9 +82,7 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3887,7 +3885,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>BOLSA ARMATODO FICHA PEQUEÑA X306 FICHAS</t>
+          <t>BOLSA ARMATODO FICHA PEQUEÃ‘A X306 FICHAS</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -7337,7 +7335,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>BOLSA ARMATODO FICHA PEQUEÑA X90 FICHAS</t>
+          <t>BOLSA ARMATODO FICHA PEQUEÃ‘A X90 FICHAS</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
@@ -7935,7 +7933,7 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>BOLSA ARMATODO FICHA PEQUEÑA X54 PIEZAS</t>
+          <t>BOLSA ARMATODO FICHA PEQUEÃ‘A X54 PIEZAS</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
@@ -7981,7 +7979,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>BOLSA ARMATODO FICHA PEQUEÑA X55 FICHAS</t>
+          <t>BOLSA ARMATODO FICHA PEQUEÃ‘A X55 FICHAS</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
@@ -8073,7 +8071,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>ARMATODOS MUÑEQUITOS 160PCS 4 MOTIVOS</t>
+          <t>ARMATODOS MUÃ‘EQUITOS 160PCS 4 MOTIVOS</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
@@ -8211,7 +8209,7 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>SET BLOQUES PEQUEÑO</t>
+          <t>SET BLOQUES PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
@@ -8947,7 +8945,7 @@
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>BOLSA ARMATODO FICHA PEQUEÑA X36 PIEZAS</t>
+          <t>BOLSA ARMATODO FICHA PEQUEÃ‘A X36 PIEZAS</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
@@ -10235,7 +10233,7 @@
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>CAJA GUITARRA NIÑA</t>
+          <t>CAJA GUITARRA NIÃ‘A</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
@@ -10971,7 +10969,7 @@
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>PIANO DELFIN PEQUEÑO 3 COLORES</t>
+          <t>PIANO DELFIN PEQUEÃ‘O 3 COLORES</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
@@ -11477,7 +11475,7 @@
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>BOLSA VAJILLA MELANINA NIÑOS</t>
+          <t>BOLSA VAJILLA MELANINA NIÃ‘OS</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
@@ -12121,7 +12119,7 @@
       </c>
       <c r="B254" s="2" t="inlineStr">
         <is>
-          <t>BURBUJERO MUÑECO AZUL</t>
+          <t>BURBUJERO MUÃ‘ECO AZUL</t>
         </is>
       </c>
       <c r="C254" s="2" t="inlineStr">
@@ -12167,7 +12165,7 @@
       </c>
       <c r="B255" s="2" t="inlineStr">
         <is>
-          <t>BURBUJERO MUÑECAS KOPP</t>
+          <t>BURBUJERO MUÃ‘ECAS KOPP</t>
         </is>
       </c>
       <c r="C255" s="2" t="inlineStr">
@@ -12811,7 +12809,7 @@
       </c>
       <c r="B269" s="2" t="inlineStr">
         <is>
-          <t>BURBUJA PITO ARAÑA</t>
+          <t>BURBUJA PITO ARAÃ‘A</t>
         </is>
       </c>
       <c r="C269" s="2" t="inlineStr">
@@ -13179,7 +13177,7 @@
       </c>
       <c r="B277" s="2" t="inlineStr">
         <is>
-          <t>ORGANIZADOR BAÑO</t>
+          <t>ORGANIZADOR BAÃ‘O</t>
         </is>
       </c>
       <c r="C277" s="2" t="inlineStr">
@@ -13363,7 +13361,7 @@
       </c>
       <c r="B281" s="2" t="inlineStr">
         <is>
-          <t>SET MAQUILLAJE PARA NIÑA UNICORNIO</t>
+          <t>SET MAQUILLAJE PARA NIÃ‘A UNICORNIO</t>
         </is>
       </c>
       <c r="C281" s="2" t="inlineStr">
@@ -14053,7 +14051,7 @@
       </c>
       <c r="B296" s="2" t="inlineStr">
         <is>
-          <t>SET DE MANILLAS MOÑO</t>
+          <t>SET DE MANILLAS MOÃ‘O</t>
         </is>
       </c>
       <c r="C296" s="2" t="inlineStr">
@@ -14651,7 +14649,7 @@
       </c>
       <c r="B309" s="2" t="inlineStr">
         <is>
-          <t>BANDEJA DE MELANINA PEQUEÑO 33CMX25CM</t>
+          <t>BANDEJA DE MELANINA PEQUEÃ‘O 33CMX25CM</t>
         </is>
       </c>
       <c r="C309" s="2" t="inlineStr">
@@ -14881,7 +14879,7 @@
       </c>
       <c r="B314" s="2" t="inlineStr">
         <is>
-          <t>BANDEJA DE MELANINA PEQUEÑO 33.5CMX26CM</t>
+          <t>BANDEJA DE MELANINA PEQUEÃ‘O 33.5CMX26CM</t>
         </is>
       </c>
       <c r="C314" s="2" t="inlineStr">
@@ -15249,7 +15247,7 @@
       </c>
       <c r="B322" s="2" t="inlineStr">
         <is>
-          <t>BOLSA PELOTA PEQUEÑA PARA GATO X9</t>
+          <t>BOLSA PELOTA PEQUEÃ‘A PARA GATO X9</t>
         </is>
       </c>
       <c r="C322" s="2" t="inlineStr">
@@ -16169,7 +16167,7 @@
       </c>
       <c r="B342" s="2" t="inlineStr">
         <is>
-          <t>LLAVERO METALICO SUPERHEROES PEQUEÑO</t>
+          <t>LLAVERO METALICO SUPERHEROES PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C342" s="2" t="inlineStr">
@@ -16445,7 +16443,7 @@
       </c>
       <c r="B348" s="2" t="inlineStr">
         <is>
-          <t>LINTERNA PEQUEÑA CAJA X 48</t>
+          <t>LINTERNA PEQUEÃ‘A CAJA X 48</t>
         </is>
       </c>
       <c r="C348" s="2" t="inlineStr">
@@ -16537,7 +16535,7 @@
       </c>
       <c r="B350" s="2" t="inlineStr">
         <is>
-          <t>LINTERNA PEQUEÑA</t>
+          <t>LINTERNA PEQUEÃ‘A</t>
         </is>
       </c>
       <c r="C350" s="2" t="inlineStr">
@@ -16583,7 +16581,7 @@
       </c>
       <c r="B351" s="2" t="inlineStr">
         <is>
-          <t>VELA NAVIDEÑA LED LUZ CALIDA 5CM ALTO X 4CM DIAMETRO</t>
+          <t>VELA NAVIDEÃ‘A LED LUZ CALIDA 5CM ALTO X 4CM DIAMETRO</t>
         </is>
       </c>
       <c r="C351" s="2" t="inlineStr">
@@ -16629,7 +16627,7 @@
       </c>
       <c r="B352" s="2" t="inlineStr">
         <is>
-          <t>VELA NAVIDEÑA LED LUZ BLANCA 5CM ALTO X 4CM DIAMETRO</t>
+          <t>VELA NAVIDEÃ‘A LED LUZ BLANCA 5CM ALTO X 4CM DIAMETRO</t>
         </is>
       </c>
       <c r="C352" s="2" t="inlineStr">
@@ -16721,7 +16719,7 @@
       </c>
       <c r="B354" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO GOTENKS SUPER SAYAJIN</t>
+          <t>MUÃ‘ECO GOTENKS SUPER SAYAJIN</t>
         </is>
       </c>
       <c r="C354" s="2" t="inlineStr">
@@ -16905,7 +16903,7 @@
       </c>
       <c r="B358" s="2" t="inlineStr">
         <is>
-          <t>COLECCION MUÑECO POKEMON</t>
+          <t>COLECCION MUÃ‘ECO POKEMON</t>
         </is>
       </c>
       <c r="C358" s="2" t="inlineStr">
@@ -16997,7 +16995,7 @@
       </c>
       <c r="B360" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO MARIO COLECCION X 6</t>
+          <t>MUÃ‘ECO MARIO COLECCION X 6</t>
         </is>
       </c>
       <c r="C360" s="2" t="inlineStr">
@@ -17043,7 +17041,7 @@
       </c>
       <c r="B361" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO OX-SATAN</t>
+          <t>MUÃ‘ECO OX-SATAN</t>
         </is>
       </c>
       <c r="C361" s="2" t="inlineStr">
@@ -17181,7 +17179,7 @@
       </c>
       <c r="B364" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO ONE PIECE BOLA DE FUEGO</t>
+          <t>MUÃ‘ECO ONE PIECE BOLA DE FUEGO</t>
         </is>
       </c>
       <c r="C364" s="2" t="inlineStr">
@@ -17365,7 +17363,7 @@
       </c>
       <c r="B368" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO PILAR</t>
+          <t>MUÃ‘ECO PILAR</t>
         </is>
       </c>
       <c r="C368" s="2" t="inlineStr">
@@ -17457,7 +17455,7 @@
       </c>
       <c r="B370" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO PILAR</t>
+          <t>MUÃ‘ECO PILAR</t>
         </is>
       </c>
       <c r="C370" s="2" t="inlineStr">
@@ -17503,7 +17501,7 @@
       </c>
       <c r="B371" s="2" t="inlineStr">
         <is>
-          <t>MUÑECOS COLLECION X 8</t>
+          <t>MUÃ‘ECOS COLLECION X 8</t>
         </is>
       </c>
       <c r="C371" s="2" t="inlineStr">
@@ -17549,7 +17547,7 @@
       </c>
       <c r="B372" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO PILAR</t>
+          <t>MUÃ‘ECO PILAR</t>
         </is>
       </c>
       <c r="C372" s="2" t="inlineStr">
@@ -17595,7 +17593,7 @@
       </c>
       <c r="B373" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO GOKU</t>
+          <t>MUÃ‘ECO GOKU</t>
         </is>
       </c>
       <c r="C373" s="2" t="inlineStr">
@@ -17687,7 +17685,7 @@
       </c>
       <c r="B375" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO ONE PIECE</t>
+          <t>MUÃ‘ECO ONE PIECE</t>
         </is>
       </c>
       <c r="C375" s="2" t="inlineStr">
@@ -17733,7 +17731,7 @@
       </c>
       <c r="B376" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO CHARMELON</t>
+          <t>MUÃ‘ECO CHARMELON</t>
         </is>
       </c>
       <c r="C376" s="2" t="inlineStr">
@@ -17779,7 +17777,7 @@
       </c>
       <c r="B377" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO IVYSAUR</t>
+          <t>MUÃ‘ECO IVYSAUR</t>
         </is>
       </c>
       <c r="C377" s="2" t="inlineStr">
@@ -17871,7 +17869,7 @@
       </c>
       <c r="B379" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO JOKER</t>
+          <t>MUÃ‘ECO JOKER</t>
         </is>
       </c>
       <c r="C379" s="2" t="inlineStr">
@@ -17963,7 +17961,7 @@
       </c>
       <c r="B381" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO HINATA BUFANDA</t>
+          <t>MUÃ‘ECO HINATA BUFANDA</t>
         </is>
       </c>
       <c r="C381" s="2" t="inlineStr">
@@ -18009,7 +18007,7 @@
       </c>
       <c r="B382" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO NARUTO BUFANDA</t>
+          <t>MUÃ‘ECO NARUTO BUFANDA</t>
         </is>
       </c>
       <c r="C382" s="2" t="inlineStr">
@@ -18193,7 +18191,7 @@
       </c>
       <c r="B386" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO MARIO GRANDE</t>
+          <t>MUÃ‘ECO MARIO GRANDE</t>
         </is>
       </c>
       <c r="C386" s="2" t="inlineStr">
@@ -18469,7 +18467,7 @@
       </c>
       <c r="B392" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO DOMA</t>
+          <t>MUÃ‘ECO DOMA</t>
         </is>
       </c>
       <c r="C392" s="2" t="inlineStr">
@@ -18561,7 +18559,7 @@
       </c>
       <c r="B394" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO POKEMON</t>
+          <t>MUÃ‘ECO POKEMON</t>
         </is>
       </c>
       <c r="C394" s="2" t="inlineStr">
@@ -18607,7 +18605,7 @@
       </c>
       <c r="B395" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO HOLLOW KNIGTH</t>
+          <t>MUÃ‘ECO HOLLOW KNIGTH</t>
         </is>
       </c>
       <c r="C395" s="2" t="inlineStr">
@@ -18653,7 +18651,7 @@
       </c>
       <c r="B396" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO AIRON MAIDEN</t>
+          <t>MUÃ‘ECO AIRON MAIDEN</t>
         </is>
       </c>
       <c r="C396" s="2" t="inlineStr">
@@ -18791,7 +18789,7 @@
       </c>
       <c r="B399" s="2" t="inlineStr">
         <is>
-          <t>MUÑECOS PLATEADOS CJ X 9 METAL DIE CAST</t>
+          <t>MUÃ‘ECOS PLATEADOS CJ X 9 METAL DIE CAST</t>
         </is>
       </c>
       <c r="C399" s="2" t="inlineStr">
@@ -22563,7 +22561,7 @@
       </c>
       <c r="B481" s="2" t="inlineStr">
         <is>
-          <t>ULA ULA PEQUEÑA 50 CM</t>
+          <t>ULA ULA PEQUEÃ‘A 50 CM</t>
         </is>
       </c>
       <c r="C481" s="2" t="inlineStr">
@@ -25369,7 +25367,7 @@
       </c>
       <c r="B542" s="2" t="inlineStr">
         <is>
-          <t>CAJA JUEGO DIDACTICO TABLA APRENDIZAJE ESPAÑOL INGLES</t>
+          <t>CAJA JUEGO DIDACTICO TABLA APRENDIZAJE ESPAÃ‘OL INGLES</t>
         </is>
       </c>
       <c r="C542" s="2" t="inlineStr">
@@ -29509,7 +29507,7 @@
       </c>
       <c r="B632" s="2" t="inlineStr">
         <is>
-          <t>FICHAS DIDACTICAS DE MULTIPLICACIÓN</t>
+          <t>FICHAS DIDACTICAS DE MULTIPLICACIÃ“N</t>
         </is>
       </c>
       <c r="C632" s="2" t="inlineStr">
@@ -30061,7 +30059,7 @@
       </c>
       <c r="B644" s="2" t="inlineStr">
         <is>
-          <t>ENCAJABLE TRIKI PEQUEÑO 14CM X 14CM</t>
+          <t>ENCAJABLE TRIKI PEQUEÃ‘O 14CM X 14CM</t>
         </is>
       </c>
       <c r="C644" s="2" t="inlineStr">
@@ -30153,7 +30151,7 @@
       </c>
       <c r="B646" s="2" t="inlineStr">
         <is>
-          <t>TABLA JUEGO DE MESA TANGRAM PEQUEÑO IMPORTADO 11CMX11CM</t>
+          <t>TABLA JUEGO DE MESA TANGRAM PEQUEÃ‘O IMPORTADO 11CMX11CM</t>
         </is>
       </c>
       <c r="C646" s="2" t="inlineStr">
@@ -31671,7 +31669,7 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>CHAMPIÑON GRANDE MASAJEADOR EN MADERA</t>
+          <t>CHAMPIÃ‘ON GRANDE MASAJEADOR EN MADERA</t>
         </is>
       </c>
       <c r="C679" s="2" t="inlineStr">
@@ -33741,7 +33739,7 @@
       </c>
       <c r="B724" s="2" t="inlineStr">
         <is>
-          <t>BINGO RULETA PEQUEÑO</t>
+          <t>BINGO RULETA PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C724" s="2" t="inlineStr">
@@ -35167,7 +35165,7 @@
       </c>
       <c r="B755" s="2" t="inlineStr">
         <is>
-          <t>PARQUES PEQUEÑO IMANADO 4-6 JUGADORES 38CM X 38CM MDF</t>
+          <t>PARQUES PEQUEÃ‘O IMANADO 4-6 JUGADORES 38CM X 38CM MDF</t>
         </is>
       </c>
       <c r="C755" s="2" t="inlineStr">
@@ -35351,7 +35349,7 @@
       </c>
       <c r="B759" s="2" t="inlineStr">
         <is>
-          <t>PARQUES Y ESCALERA VIAJERO PEQUEÑO CON BORDE DOBLAR EN 2</t>
+          <t>PARQUES Y ESCALERA VIAJERO PEQUEÃ‘O CON BORDE DOBLAR EN 2</t>
         </is>
       </c>
       <c r="C759" s="2" t="inlineStr">
@@ -35489,7 +35487,7 @@
       </c>
       <c r="B762" s="2" t="inlineStr">
         <is>
-          <t>PARQUES 4 6 PUESTOS VIAJERO PEQUEÑO CON BORDE DOBLAR EN 2</t>
+          <t>PARQUES 4 6 PUESTOS VIAJERO PEQUEÃ‘O CON BORDE DOBLAR EN 2</t>
         </is>
       </c>
       <c r="C762" s="2" t="inlineStr">
@@ -37007,7 +37005,7 @@
       </c>
       <c r="B795" s="2" t="inlineStr">
         <is>
-          <t>PARQUES PEQUEÑO SENCILLO 4-6 JUGADORES 38CM X 38CM PINO</t>
+          <t>PARQUES PEQUEÃ‘O SENCILLO 4-6 JUGADORES 38CM X 38CM PINO</t>
         </is>
       </c>
       <c r="C795" s="2" t="inlineStr">
@@ -37283,7 +37281,7 @@
       </c>
       <c r="B801" s="2" t="inlineStr">
         <is>
-          <t>CENTRO DERECHA IZQUIERDA PEQUEÑO</t>
+          <t>CENTRO DERECHA IZQUIERDA PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C801" s="2" t="inlineStr">
@@ -37651,7 +37649,7 @@
       </c>
       <c r="B809" s="2" t="inlineStr">
         <is>
-          <t>CAJA JUEGO DE MESA CAJA 8 LEÑOS MADERA</t>
+          <t>CAJA JUEGO DE MESA CAJA 8 LEÃ‘OS MADERA</t>
         </is>
       </c>
       <c r="C809" s="2" t="inlineStr">
@@ -37835,7 +37833,7 @@
       </c>
       <c r="B813" s="2" t="inlineStr">
         <is>
-          <t>DOMINO SASPIADO PEQUEÑO</t>
+          <t>DOMINO SASPIADO PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C813" s="2" t="inlineStr">
@@ -38203,7 +38201,7 @@
       </c>
       <c r="B821" s="2" t="inlineStr">
         <is>
-          <t>POKER LETRA PEQUEÑA PLASTICO SEMIORIGINAL</t>
+          <t>POKER LETRA PEQUEÃ‘A PLASTICO SEMIORIGINAL</t>
         </is>
       </c>
       <c r="C821" s="2" t="inlineStr">
@@ -38295,7 +38293,7 @@
       </c>
       <c r="B823" s="2" t="inlineStr">
         <is>
-          <t>AJEDREZ 3 EN 1 SERIES CAJA BLANCA PEQUEÑO</t>
+          <t>AJEDREZ 3 EN 1 SERIES CAJA BLANCA PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C823" s="2" t="inlineStr">
@@ -38709,7 +38707,7 @@
       </c>
       <c r="B832" s="2" t="inlineStr">
         <is>
-          <t>POKER LETRA PEQUEÑA SEMIORIGINAL</t>
+          <t>POKER LETRA PEQUEÃ‘A SEMIORIGINAL</t>
         </is>
       </c>
       <c r="C832" s="2" t="inlineStr">
@@ -38893,7 +38891,7 @@
       </c>
       <c r="B836" s="2" t="inlineStr">
         <is>
-          <t>JUEGO DE GESTOS PEQUEÑO CAJA CARTON</t>
+          <t>JUEGO DE GESTOS PEQUEÃ‘O CAJA CARTON</t>
         </is>
       </c>
       <c r="C836" s="2" t="inlineStr">
@@ -39031,7 +39029,7 @@
       </c>
       <c r="B839" s="2" t="inlineStr">
         <is>
-          <t>BARAJA ESPAÑOLA BLANCO ORIGINAL</t>
+          <t>BARAJA ESPAÃ‘OLA BLANCO ORIGINAL</t>
         </is>
       </c>
       <c r="C839" s="2" t="inlineStr">
@@ -39307,7 +39305,7 @@
       </c>
       <c r="B845" s="2" t="inlineStr">
         <is>
-          <t>DOMINO FICHA PEQUEÑA ESTUCHE</t>
+          <t>DOMINO FICHA PEQUEÃ‘A ESTUCHE</t>
         </is>
       </c>
       <c r="C845" s="2" t="inlineStr">
@@ -39813,7 +39811,7 @@
       </c>
       <c r="B856" s="2" t="inlineStr">
         <is>
-          <t>CAJA BARAJA ESPAÑOLA BLANCO SEMIORIGINAL</t>
+          <t>CAJA BARAJA ESPAÃ‘OLA BLANCO SEMIORIGINAL</t>
         </is>
       </c>
       <c r="C856" s="2" t="inlineStr">
@@ -39951,7 +39949,7 @@
       </c>
       <c r="B859" s="2" t="inlineStr">
         <is>
-          <t>JENGA PEQUEÑO CAJA AZUL 15CM*5CM</t>
+          <t>JENGA PEQUEÃ‘O CAJA AZUL 15CM*5CM</t>
         </is>
       </c>
       <c r="C859" s="2" t="inlineStr">
@@ -39997,7 +39995,7 @@
       </c>
       <c r="B860" s="2" t="inlineStr">
         <is>
-          <t>BARAJA ESPAÑOLA BLANCO SEMIORIGINAL</t>
+          <t>BARAJA ESPAÃ‘OLA BLANCO SEMIORIGINAL</t>
         </is>
       </c>
       <c r="C860" s="2" t="inlineStr">
@@ -40089,7 +40087,7 @@
       </c>
       <c r="B862" s="2" t="inlineStr">
         <is>
-          <t>CARTA ESPAÑOLA VERDE 10.5CM X 7CM</t>
+          <t>CARTA ESPAÃ‘OLA VERDE 10.5CM X 7CM</t>
         </is>
       </c>
       <c r="C862" s="2" t="inlineStr">
@@ -40595,7 +40593,7 @@
       </c>
       <c r="B873" s="2" t="inlineStr">
         <is>
-          <t>CARTA ESPAÑOLA BLANCO SENCILLO 9.9CMX7.0CM</t>
+          <t>CARTA ESPAÃ‘OLA BLANCO SENCILLO 9.9CMX7.0CM</t>
         </is>
       </c>
       <c r="C873" s="2" t="inlineStr">
@@ -40825,7 +40823,7 @@
       </c>
       <c r="B878" s="2" t="inlineStr">
         <is>
-          <t>DADO CRISTAL PEQUEÑO X 50</t>
+          <t>DADO CRISTAL PEQUEÃ‘O X 50</t>
         </is>
       </c>
       <c r="C878" s="2" t="inlineStr">
@@ -41331,7 +41329,7 @@
       </c>
       <c r="B889" s="2" t="inlineStr">
         <is>
-          <t>CASA PARA MUÑECA ARMABLE CAJA 83CM*52CM</t>
+          <t>CASA PARA MUÃ‘ECA ARMABLE CAJA 83CM*52CM</t>
         </is>
       </c>
       <c r="C889" s="2" t="inlineStr">
@@ -41469,7 +41467,7 @@
       </c>
       <c r="B892" s="2" t="inlineStr">
         <is>
-          <t>CASA MUÑECA ARMABLE X 157PCS</t>
+          <t>CASA MUÃ‘ECA ARMABLE X 157PCS</t>
         </is>
       </c>
       <c r="C892" s="2" t="inlineStr">
@@ -42067,7 +42065,7 @@
       </c>
       <c r="B905" s="2" t="inlineStr">
         <is>
-          <t>CARRO CONTROL REMOTO NIÑA ROSADO</t>
+          <t>CARRO CONTROL REMOTO NIÃ‘A ROSADO</t>
         </is>
       </c>
       <c r="C905" s="2" t="inlineStr">
@@ -42343,7 +42341,7 @@
       </c>
       <c r="B911" s="2" t="inlineStr">
         <is>
-          <t>CAJA REGISTRADORA CON ACCESORIOS (PILAS) NIÑA</t>
+          <t>CAJA REGISTRADORA CON ACCESORIOS (PILAS) NIÃ‘A</t>
         </is>
       </c>
       <c r="C911" s="2" t="inlineStr">
@@ -43493,7 +43491,7 @@
       </c>
       <c r="B936" s="2" t="inlineStr">
         <is>
-          <t>COCHE MOISES PARA MUÑECA GRANDE</t>
+          <t>COCHE MOISES PARA MUÃ‘ECA GRANDE</t>
         </is>
       </c>
       <c r="C936" s="2" t="inlineStr">
@@ -43539,7 +43537,7 @@
       </c>
       <c r="B937" s="2" t="inlineStr">
         <is>
-          <t>CAJA COLECCIÓN SAFARI ANIMALES SELVA</t>
+          <t>CAJA COLECCIÃ“N SAFARI ANIMALES SELVA</t>
         </is>
       </c>
       <c r="C937" s="2" t="inlineStr">
@@ -44873,7 +44871,7 @@
       </c>
       <c r="B966" s="2" t="inlineStr">
         <is>
-          <t>CARRO NIÑERA SURTIDA</t>
+          <t>CARRO NIÃ‘ERA SURTIDA</t>
         </is>
       </c>
       <c r="C966" s="2" t="inlineStr">
@@ -45011,7 +45009,7 @@
       </c>
       <c r="B969" s="2" t="inlineStr">
         <is>
-          <t>COCHE MOISES PARA MUÑECAS PQ</t>
+          <t>COCHE MOISES PARA MUÃ‘ECAS PQ</t>
         </is>
       </c>
       <c r="C969" s="2" t="inlineStr">
@@ -45149,7 +45147,7 @@
       </c>
       <c r="B972" s="2" t="inlineStr">
         <is>
-          <t>MUÑECA PILA LUZ SONIDO CJ ALICE PRINCESS</t>
+          <t>MUÃ‘ECA PILA LUZ SONIDO CJ ALICE PRINCESS</t>
         </is>
       </c>
       <c r="C972" s="2" t="inlineStr">
@@ -45563,7 +45561,7 @@
       </c>
       <c r="B981" s="2" t="inlineStr">
         <is>
-          <t>COCHE PARA MUÑECAS MD</t>
+          <t>COCHE PARA MUÃ‘ECAS MD</t>
         </is>
       </c>
       <c r="C981" s="2" t="inlineStr">
@@ -45747,7 +45745,7 @@
       </c>
       <c r="B985" s="2" t="inlineStr">
         <is>
-          <t>GUITARRA PEQUEÑA LA CAUCANA EN MADERA</t>
+          <t>GUITARRA PEQUEÃ‘A LA CAUCANA EN MADERA</t>
         </is>
       </c>
       <c r="C985" s="2" t="inlineStr">
@@ -46391,7 +46389,7 @@
       </c>
       <c r="B999" s="2" t="inlineStr">
         <is>
-          <t>MUÑECA CRESPA</t>
+          <t>MUÃ‘ECA CRESPA</t>
         </is>
       </c>
       <c r="C999" s="2" t="inlineStr">
@@ -46575,7 +46573,7 @@
       </c>
       <c r="B1003" s="2" t="inlineStr">
         <is>
-          <t>MUÑECA BEBE CRESPA EN CAJA</t>
+          <t>MUÃ‘ECA BEBE CRESPA EN CAJA</t>
         </is>
       </c>
       <c r="C1003" s="2" t="inlineStr">
@@ -47311,7 +47309,7 @@
       </c>
       <c r="B1019" s="2" t="inlineStr">
         <is>
-          <t>MULA NIÑERA CON CARROS 2 COLORES</t>
+          <t>MULA NIÃ‘ERA CON CARROS 2 COLORES</t>
         </is>
       </c>
       <c r="C1019" s="2" t="inlineStr">
@@ -47357,7 +47355,7 @@
       </c>
       <c r="B1020" s="2" t="inlineStr">
         <is>
-          <t>CARRO NIÑERA CON DINOSAURIO</t>
+          <t>CARRO NIÃ‘ERA CON DINOSAURIO</t>
         </is>
       </c>
       <c r="C1020" s="2" t="inlineStr">
@@ -47495,7 +47493,7 @@
       </c>
       <c r="B1023" s="2" t="inlineStr">
         <is>
-          <t>MUÑECA AFRO SET</t>
+          <t>MUÃ‘ECA AFRO SET</t>
         </is>
       </c>
       <c r="C1023" s="2" t="inlineStr">
@@ -47771,7 +47769,7 @@
       </c>
       <c r="B1029" s="2" t="inlineStr">
         <is>
-          <t>DINOSAURIO ZAZA DE PILA 5 DISEÑOS</t>
+          <t>DINOSAURIO ZAZA DE PILA 5 DISEÃ‘OS</t>
         </is>
       </c>
       <c r="C1029" s="2" t="inlineStr">
@@ -48599,7 +48597,7 @@
       </c>
       <c r="B1047" s="2" t="inlineStr">
         <is>
-          <t>MUÑECA CRESPA PEQUEÑA</t>
+          <t>MUÃ‘ECA CRESPA PEQUEÃ‘A</t>
         </is>
       </c>
       <c r="C1047" s="2" t="inlineStr">
@@ -48967,7 +48965,7 @@
       </c>
       <c r="B1055" s="2" t="inlineStr">
         <is>
-          <t>VAJILLA TULA TETERA PEQUEÑA</t>
+          <t>VAJILLA TULA TETERA PEQUEÃ‘A</t>
         </is>
       </c>
       <c r="C1055" s="2" t="inlineStr">
@@ -49059,7 +49057,7 @@
       </c>
       <c r="B1057" s="2" t="inlineStr">
         <is>
-          <t>CAJA LANZADARDOS 3 SOFTGUN PEQUEÑO 2 COLORES</t>
+          <t>CAJA LANZADARDOS 3 SOFTGUN PEQUEÃ‘O 2 COLORES</t>
         </is>
       </c>
       <c r="C1057" s="2" t="inlineStr">
@@ -49933,7 +49931,7 @@
       </c>
       <c r="B1076" s="2" t="inlineStr">
         <is>
-          <t>CARTON GUANTE LANZADARDOS ARAÑA</t>
+          <t>CARTON GUANTE LANZADARDOS ARAÃ‘A</t>
         </is>
       </c>
       <c r="C1076" s="2" t="inlineStr">
@@ -50209,7 +50207,7 @@
       </c>
       <c r="B1082" s="2" t="inlineStr">
         <is>
-          <t>SET ESMALTE PARA NIÑAS X5</t>
+          <t>SET ESMALTE PARA NIÃ‘AS X5</t>
         </is>
       </c>
       <c r="C1082" s="2" t="inlineStr">
@@ -50393,7 +50391,7 @@
       </c>
       <c r="B1086" s="2" t="inlineStr">
         <is>
-          <t>MUÑECO BEBE</t>
+          <t>MUÃ‘ECO BEBE</t>
         </is>
       </c>
       <c r="C1086" s="2" t="inlineStr">
@@ -50669,7 +50667,7 @@
       </c>
       <c r="B1092" s="2" t="inlineStr">
         <is>
-          <t>BEBE CON BAÑER EN BOLSA</t>
+          <t>BEBE CON BAÃ‘ER EN BOLSA</t>
         </is>
       </c>
       <c r="C1092" s="2" t="inlineStr">
@@ -50853,7 +50851,7 @@
       </c>
       <c r="B1096" s="2" t="inlineStr">
         <is>
-          <t>BOLSA MASCARA MUÑECO CON LUZ</t>
+          <t>BOLSA MASCARA MUÃ‘ECO CON LUZ</t>
         </is>
       </c>
       <c r="C1096" s="2" t="inlineStr">
@@ -51313,7 +51311,7 @@
       </c>
       <c r="B1106" s="2" t="inlineStr">
         <is>
-          <t>TROMPO MADERA X12 PEQUEÑO</t>
+          <t>TROMPO MADERA X12 PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1106" s="2" t="inlineStr">
@@ -51405,7 +51403,7 @@
       </c>
       <c r="B1108" s="2" t="inlineStr">
         <is>
-          <t>CAJA MUÑECA LENTEJUELAS</t>
+          <t>CAJA MUÃ‘ECA LENTEJUELAS</t>
         </is>
       </c>
       <c r="C1108" s="2" t="inlineStr">
@@ -51497,7 +51495,7 @@
       </c>
       <c r="B1110" s="2" t="inlineStr">
         <is>
-          <t>BAÑERA CON BEBE Y ACCESORIOS EN BOLSA</t>
+          <t>BAÃ‘ERA CON BEBE Y ACCESORIOS EN BOLSA</t>
         </is>
       </c>
       <c r="C1110" s="2" t="inlineStr">
@@ -51957,7 +51955,7 @@
       </c>
       <c r="B1120" s="2" t="inlineStr">
         <is>
-          <t>AVION DE IMPULSO LUZ Y SONIDO EN BOLSA PEQUEÑO</t>
+          <t>AVION DE IMPULSO LUZ Y SONIDO EN BOLSA PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1120" s="2" t="inlineStr">
@@ -52233,7 +52231,7 @@
       </c>
       <c r="B1126" s="2" t="inlineStr">
         <is>
-          <t>BAÑERA CON BEBE Y ACCESORIOS EN BOLSA DOS COLORES</t>
+          <t>BAÃ‘ERA CON BEBE Y ACCESORIOS EN BOLSA DOS COLORES</t>
         </is>
       </c>
       <c r="C1126" s="2" t="inlineStr">
@@ -52555,7 +52553,7 @@
       </c>
       <c r="B1133" s="2" t="inlineStr">
         <is>
-          <t>MULA NIÑERA 3 COLORES</t>
+          <t>MULA NIÃ‘ERA 3 COLORES</t>
         </is>
       </c>
       <c r="C1133" s="2" t="inlineStr">
@@ -53199,7 +53197,7 @@
       </c>
       <c r="B1147" s="2" t="inlineStr">
         <is>
-          <t>BOLSITO LOL MUÑECA Y ACCESORIOS</t>
+          <t>BOLSITO LOL MUÃ‘ECA Y ACCESORIOS</t>
         </is>
       </c>
       <c r="C1147" s="2" t="inlineStr">
@@ -53751,7 +53749,7 @@
       </c>
       <c r="B1159" s="2" t="inlineStr">
         <is>
-          <t>CAJA KIT DE UÑAS CON CIRCULO</t>
+          <t>CAJA KIT DE UÃ‘AS CON CIRCULO</t>
         </is>
       </c>
       <c r="C1159" s="2" t="inlineStr">
@@ -56373,7 +56371,7 @@
       </c>
       <c r="B1216" s="2" t="inlineStr">
         <is>
-          <t>BOLSO OSO CARIÑOSITO</t>
+          <t>BOLSO OSO CARIÃ‘OSITO</t>
         </is>
       </c>
       <c r="C1216" s="2" t="inlineStr">
@@ -56787,7 +56785,7 @@
       </c>
       <c r="B1225" s="2" t="inlineStr">
         <is>
-          <t>LLAVERO CAPIBARA PELUCHE PEQUEÑO 6 MOTIVOS</t>
+          <t>LLAVERO CAPIBARA PELUCHE PEQUEÃ‘O 6 MOTIVOS</t>
         </is>
       </c>
       <c r="C1225" s="2" t="inlineStr">
@@ -57344,7 +57342,7 @@
       </c>
       <c r="C1237" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1237" s="3" t="n">
@@ -57390,7 +57388,7 @@
       </c>
       <c r="C1238" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1238" s="3" t="n">
@@ -57436,7 +57434,7 @@
       </c>
       <c r="C1239" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1239" s="3" t="n">
@@ -57482,7 +57480,7 @@
       </c>
       <c r="C1240" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1240" s="3" t="n">
@@ -57528,7 +57526,7 @@
       </c>
       <c r="C1241" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1241" s="3" t="n">
@@ -57574,7 +57572,7 @@
       </c>
       <c r="C1242" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1242" s="3" t="n">
@@ -57620,7 +57618,7 @@
       </c>
       <c r="C1243" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1243" s="3" t="n">
@@ -57666,7 +57664,7 @@
       </c>
       <c r="C1244" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1244" s="3" t="n">
@@ -57712,7 +57710,7 @@
       </c>
       <c r="C1245" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1245" s="3" t="n">
@@ -57758,7 +57756,7 @@
       </c>
       <c r="C1246" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1246" s="3" t="n">
@@ -57804,7 +57802,7 @@
       </c>
       <c r="C1247" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1247" s="3" t="n">
@@ -57845,12 +57843,12 @@
       </c>
       <c r="B1248" s="2" t="inlineStr">
         <is>
-          <t>CARTON HOMBRE ARAÑA CON LUCES Y SONIDO GRANDE</t>
+          <t>CARTON HOMBRE ARAÃ‘A CON LUCES Y SONIDO GRANDE</t>
         </is>
       </c>
       <c r="C1248" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1248" s="3" t="n">
@@ -57896,7 +57894,7 @@
       </c>
       <c r="C1249" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1249" s="3" t="n">
@@ -57942,7 +57940,7 @@
       </c>
       <c r="C1250" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1250" s="3" t="n">
@@ -57988,7 +57986,7 @@
       </c>
       <c r="C1251" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1251" s="3" t="n">
@@ -58034,7 +58032,7 @@
       </c>
       <c r="C1252" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1252" s="3" t="n">
@@ -58080,7 +58078,7 @@
       </c>
       <c r="C1253" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1253" s="3" t="n">
@@ -58126,7 +58124,7 @@
       </c>
       <c r="C1254" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1254" s="3" t="n">
@@ -58172,7 +58170,7 @@
       </c>
       <c r="C1255" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1255" s="3" t="n">
@@ -58218,7 +58216,7 @@
       </c>
       <c r="C1256" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1256" s="3" t="n">
@@ -58264,7 +58262,7 @@
       </c>
       <c r="C1257" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1257" s="3" t="n">
@@ -58310,7 +58308,7 @@
       </c>
       <c r="C1258" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1258" s="3" t="n">
@@ -58356,7 +58354,7 @@
       </c>
       <c r="C1259" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1259" s="3" t="n">
@@ -58402,7 +58400,7 @@
       </c>
       <c r="C1260" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1260" s="3" t="n">
@@ -58448,7 +58446,7 @@
       </c>
       <c r="C1261" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1261" s="3" t="n">
@@ -58494,7 +58492,7 @@
       </c>
       <c r="C1262" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1262" s="3" t="n">
@@ -58540,7 +58538,7 @@
       </c>
       <c r="C1263" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1263" s="3" t="n">
@@ -58586,7 +58584,7 @@
       </c>
       <c r="C1264" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1264" s="3" t="n">
@@ -58632,7 +58630,7 @@
       </c>
       <c r="C1265" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1265" s="3" t="n">
@@ -58678,7 +58676,7 @@
       </c>
       <c r="C1266" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1266" s="3" t="n">
@@ -58724,7 +58722,7 @@
       </c>
       <c r="C1267" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1267" s="3" t="n">
@@ -58770,7 +58768,7 @@
       </c>
       <c r="C1268" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1268" s="3" t="n">
@@ -58816,7 +58814,7 @@
       </c>
       <c r="C1269" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1269" s="3" t="n">
@@ -58862,7 +58860,7 @@
       </c>
       <c r="C1270" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1270" s="3" t="n">
@@ -58908,7 +58906,7 @@
       </c>
       <c r="C1271" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1271" s="3" t="n">
@@ -58954,7 +58952,7 @@
       </c>
       <c r="C1272" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1272" s="3" t="n">
@@ -59000,7 +58998,7 @@
       </c>
       <c r="C1273" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1273" s="3" t="n">
@@ -59046,7 +59044,7 @@
       </c>
       <c r="C1274" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1274" s="3" t="n">
@@ -59092,7 +59090,7 @@
       </c>
       <c r="C1275" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1275" s="3" t="n">
@@ -59138,7 +59136,7 @@
       </c>
       <c r="C1276" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1276" s="3" t="n">
@@ -59184,7 +59182,7 @@
       </c>
       <c r="C1277" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1277" s="3" t="n">
@@ -59230,7 +59228,7 @@
       </c>
       <c r="C1278" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1278" s="3" t="n">
@@ -59276,7 +59274,7 @@
       </c>
       <c r="C1279" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1279" s="3" t="n">
@@ -59322,7 +59320,7 @@
       </c>
       <c r="C1280" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1280" s="3" t="n">
@@ -59368,7 +59366,7 @@
       </c>
       <c r="C1281" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1281" s="3" t="n">
@@ -59414,7 +59412,7 @@
       </c>
       <c r="C1282" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1282" s="3" t="n">
@@ -59460,7 +59458,7 @@
       </c>
       <c r="C1283" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1283" s="3" t="n">
@@ -59506,7 +59504,7 @@
       </c>
       <c r="C1284" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1284" s="3" t="n">
@@ -59552,7 +59550,7 @@
       </c>
       <c r="C1285" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1285" s="3" t="n">
@@ -59598,7 +59596,7 @@
       </c>
       <c r="C1286" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1286" s="3" t="n">
@@ -59644,7 +59642,7 @@
       </c>
       <c r="C1287" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1287" s="3" t="n">
@@ -59690,7 +59688,7 @@
       </c>
       <c r="C1288" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1288" s="3" t="n">
@@ -59736,7 +59734,7 @@
       </c>
       <c r="C1289" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1289" s="3" t="n">
@@ -59782,7 +59780,7 @@
       </c>
       <c r="C1290" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1290" s="3" t="n">
@@ -59828,7 +59826,7 @@
       </c>
       <c r="C1291" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1291" s="3" t="n">
@@ -59874,7 +59872,7 @@
       </c>
       <c r="C1292" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1292" s="3" t="n">
@@ -59920,7 +59918,7 @@
       </c>
       <c r="C1293" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1293" s="3" t="n">
@@ -59966,7 +59964,7 @@
       </c>
       <c r="C1294" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1294" s="3" t="n">
@@ -60012,7 +60010,7 @@
       </c>
       <c r="C1295" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1295" s="3" t="n">
@@ -60058,7 +60056,7 @@
       </c>
       <c r="C1296" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1296" s="3" t="n">
@@ -60104,7 +60102,7 @@
       </c>
       <c r="C1297" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1297" s="3" t="n">
@@ -60150,7 +60148,7 @@
       </c>
       <c r="C1298" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1298" s="3" t="n">
@@ -60196,7 +60194,7 @@
       </c>
       <c r="C1299" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1299" s="3" t="n">
@@ -60242,7 +60240,7 @@
       </c>
       <c r="C1300" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1300" s="3" t="n">
@@ -60288,7 +60286,7 @@
       </c>
       <c r="C1301" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1301" s="3" t="n">
@@ -60334,7 +60332,7 @@
       </c>
       <c r="C1302" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1302" s="3" t="n">
@@ -60380,7 +60378,7 @@
       </c>
       <c r="C1303" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1303" s="3" t="n">
@@ -60426,7 +60424,7 @@
       </c>
       <c r="C1304" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1304" s="3" t="n">
@@ -60472,7 +60470,7 @@
       </c>
       <c r="C1305" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1305" s="3" t="n">
@@ -60518,7 +60516,7 @@
       </c>
       <c r="C1306" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1306" s="3" t="n">
@@ -60564,7 +60562,7 @@
       </c>
       <c r="C1307" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1307" s="3" t="n">
@@ -60610,7 +60608,7 @@
       </c>
       <c r="C1308" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1308" s="3" t="n">
@@ -60656,7 +60654,7 @@
       </c>
       <c r="C1309" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1309" s="3" t="n">
@@ -60702,7 +60700,7 @@
       </c>
       <c r="C1310" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1310" s="3" t="n">
@@ -60748,7 +60746,7 @@
       </c>
       <c r="C1311" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1311" s="3" t="n">
@@ -60794,7 +60792,7 @@
       </c>
       <c r="C1312" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1312" s="3" t="n">
@@ -60840,7 +60838,7 @@
       </c>
       <c r="C1313" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1313" s="3" t="n">
@@ -60886,7 +60884,7 @@
       </c>
       <c r="C1314" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1314" s="3" t="n">
@@ -60932,7 +60930,7 @@
       </c>
       <c r="C1315" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1315" s="3" t="n">
@@ -60978,7 +60976,7 @@
       </c>
       <c r="C1316" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1316" s="3" t="n">
@@ -61024,7 +61022,7 @@
       </c>
       <c r="C1317" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1317" s="3" t="n">
@@ -61070,7 +61068,7 @@
       </c>
       <c r="C1318" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1318" s="3" t="n">
@@ -61116,7 +61114,7 @@
       </c>
       <c r="C1319" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1319" s="3" t="n">
@@ -61162,7 +61160,7 @@
       </c>
       <c r="C1320" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1320" s="3" t="n">
@@ -61208,7 +61206,7 @@
       </c>
       <c r="C1321" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1321" s="3" t="n">
@@ -61254,7 +61252,7 @@
       </c>
       <c r="C1322" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1322" s="3" t="n">
@@ -61300,7 +61298,7 @@
       </c>
       <c r="C1323" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1323" s="3" t="n">
@@ -61346,7 +61344,7 @@
       </c>
       <c r="C1324" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1324" s="3" t="n">
@@ -61392,7 +61390,7 @@
       </c>
       <c r="C1325" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1325" s="3" t="n">
@@ -61438,7 +61436,7 @@
       </c>
       <c r="C1326" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1326" s="3" t="n">
@@ -61484,7 +61482,7 @@
       </c>
       <c r="C1327" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1327" s="3" t="n">
@@ -61530,7 +61528,7 @@
       </c>
       <c r="C1328" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1328" s="3" t="n">
@@ -61576,7 +61574,7 @@
       </c>
       <c r="C1329" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1329" s="3" t="n">
@@ -61622,7 +61620,7 @@
       </c>
       <c r="C1330" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1330" s="3" t="n">
@@ -61668,7 +61666,7 @@
       </c>
       <c r="C1331" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1331" s="3" t="n">
@@ -61714,7 +61712,7 @@
       </c>
       <c r="C1332" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1332" s="3" t="n">
@@ -61760,7 +61758,7 @@
       </c>
       <c r="C1333" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1333" s="3" t="n">
@@ -61806,7 +61804,7 @@
       </c>
       <c r="C1334" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1334" s="3" t="n">
@@ -61852,7 +61850,7 @@
       </c>
       <c r="C1335" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1335" s="3" t="n">
@@ -61898,7 +61896,7 @@
       </c>
       <c r="C1336" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1336" s="3" t="n">
@@ -61944,7 +61942,7 @@
       </c>
       <c r="C1337" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1337" s="3" t="n">
@@ -61990,7 +61988,7 @@
       </c>
       <c r="C1338" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1338" s="3" t="n">
@@ -62036,7 +62034,7 @@
       </c>
       <c r="C1339" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1339" s="3" t="n">
@@ -62082,7 +62080,7 @@
       </c>
       <c r="C1340" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1340" s="3" t="n">
@@ -62128,7 +62126,7 @@
       </c>
       <c r="C1341" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1341" s="3" t="n">
@@ -62174,7 +62172,7 @@
       </c>
       <c r="C1342" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1342" s="3" t="n">
@@ -62220,7 +62218,7 @@
       </c>
       <c r="C1343" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1343" s="3" t="n">
@@ -62266,7 +62264,7 @@
       </c>
       <c r="C1344" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1344" s="3" t="n">
@@ -62312,7 +62310,7 @@
       </c>
       <c r="C1345" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1345" s="3" t="n">
@@ -62358,7 +62356,7 @@
       </c>
       <c r="C1346" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1346" s="3" t="n">
@@ -62404,7 +62402,7 @@
       </c>
       <c r="C1347" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1347" s="3" t="n">
@@ -62450,7 +62448,7 @@
       </c>
       <c r="C1348" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1348" s="3" t="n">
@@ -62496,7 +62494,7 @@
       </c>
       <c r="C1349" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1349" s="3" t="n">
@@ -62542,7 +62540,7 @@
       </c>
       <c r="C1350" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1350" s="3" t="n">
@@ -62588,7 +62586,7 @@
       </c>
       <c r="C1351" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1351" s="3" t="n">
@@ -62634,7 +62632,7 @@
       </c>
       <c r="C1352" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1352" s="3" t="n">
@@ -62680,7 +62678,7 @@
       </c>
       <c r="C1353" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1353" s="3" t="n">
@@ -62726,7 +62724,7 @@
       </c>
       <c r="C1354" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1354" s="3" t="n">
@@ -62772,7 +62770,7 @@
       </c>
       <c r="C1355" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1355" s="3" t="n">
@@ -62818,7 +62816,7 @@
       </c>
       <c r="C1356" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1356" s="3" t="n">
@@ -62864,7 +62862,7 @@
       </c>
       <c r="C1357" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1357" s="3" t="n">
@@ -62910,7 +62908,7 @@
       </c>
       <c r="C1358" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1358" s="3" t="n">
@@ -62956,7 +62954,7 @@
       </c>
       <c r="C1359" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1359" s="3" t="n">
@@ -63002,7 +63000,7 @@
       </c>
       <c r="C1360" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1360" s="3" t="n">
@@ -63048,7 +63046,7 @@
       </c>
       <c r="C1361" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1361" s="3" t="n">
@@ -63094,7 +63092,7 @@
       </c>
       <c r="C1362" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1362" s="3" t="n">
@@ -63140,7 +63138,7 @@
       </c>
       <c r="C1363" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1363" s="3" t="n">
@@ -63186,7 +63184,7 @@
       </c>
       <c r="C1364" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1364" s="3" t="n">
@@ -63232,7 +63230,7 @@
       </c>
       <c r="C1365" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1365" s="3" t="n">
@@ -63278,7 +63276,7 @@
       </c>
       <c r="C1366" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1366" s="3" t="n">
@@ -63324,7 +63322,7 @@
       </c>
       <c r="C1367" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1367" s="3" t="n">
@@ -63370,7 +63368,7 @@
       </c>
       <c r="C1368" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1368" s="3" t="n">
@@ -63416,7 +63414,7 @@
       </c>
       <c r="C1369" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1369" s="3" t="n">
@@ -63462,7 +63460,7 @@
       </c>
       <c r="C1370" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1370" s="3" t="n">
@@ -63508,7 +63506,7 @@
       </c>
       <c r="C1371" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1371" s="3" t="n">
@@ -63554,7 +63552,7 @@
       </c>
       <c r="C1372" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1372" s="3" t="n">
@@ -63600,7 +63598,7 @@
       </c>
       <c r="C1373" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1373" s="3" t="n">
@@ -63646,7 +63644,7 @@
       </c>
       <c r="C1374" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1374" s="3" t="n">
@@ -63692,7 +63690,7 @@
       </c>
       <c r="C1375" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1375" s="3" t="n">
@@ -63738,7 +63736,7 @@
       </c>
       <c r="C1376" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1376" s="3" t="n">
@@ -63784,7 +63782,7 @@
       </c>
       <c r="C1377" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1377" s="3" t="n">
@@ -63825,12 +63823,12 @@
       </c>
       <c r="B1378" s="2" t="inlineStr">
         <is>
-          <t>SET BILLETERA RELOJ Y GAFAS MUÑECOS</t>
+          <t>SET BILLETERA RELOJ Y GAFAS MUÃ‘ECOS</t>
         </is>
       </c>
       <c r="C1378" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1378" s="3" t="n">
@@ -63876,7 +63874,7 @@
       </c>
       <c r="C1379" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1379" s="3" t="n">
@@ -63922,7 +63920,7 @@
       </c>
       <c r="C1380" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1380" s="3" t="n">
@@ -63968,7 +63966,7 @@
       </c>
       <c r="C1381" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1381" s="3" t="n">
@@ -64014,7 +64012,7 @@
       </c>
       <c r="C1382" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1382" s="3" t="n">
@@ -64060,7 +64058,7 @@
       </c>
       <c r="C1383" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1383" s="3" t="n">
@@ -64106,7 +64104,7 @@
       </c>
       <c r="C1384" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1384" s="3" t="n">
@@ -64147,12 +64145,12 @@
       </c>
       <c r="B1385" s="2" t="inlineStr">
         <is>
-          <t>AVION MUÑEQUITO CANINO DE IMPULSO</t>
+          <t>AVION MUÃ‘EQUITO CANINO DE IMPULSO</t>
         </is>
       </c>
       <c r="C1385" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1385" s="3" t="n">
@@ -64198,7 +64196,7 @@
       </c>
       <c r="C1386" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1386" s="3" t="n">
@@ -64244,7 +64242,7 @@
       </c>
       <c r="C1387" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1387" s="3" t="n">
@@ -64290,7 +64288,7 @@
       </c>
       <c r="C1388" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1388" s="3" t="n">
@@ -64336,7 +64334,7 @@
       </c>
       <c r="C1389" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1389" s="3" t="n">
@@ -64377,12 +64375,12 @@
       </c>
       <c r="B1390" s="2" t="inlineStr">
         <is>
-          <t>AVION MUÑEQUITOS DE IMPULSO</t>
+          <t>AVION MUÃ‘EQUITOS DE IMPULSO</t>
         </is>
       </c>
       <c r="C1390" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1390" s="3" t="n">
@@ -64423,12 +64421,12 @@
       </c>
       <c r="B1391" s="2" t="inlineStr">
         <is>
-          <t>SET MUÑECOS GUERREROS</t>
+          <t>SET MUÃ‘ECOS GUERREROS</t>
         </is>
       </c>
       <c r="C1391" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1391" s="3" t="n">
@@ -64474,7 +64472,7 @@
       </c>
       <c r="C1392" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1392" s="3" t="n">
@@ -64520,7 +64518,7 @@
       </c>
       <c r="C1393" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1393" s="3" t="n">
@@ -64566,7 +64564,7 @@
       </c>
       <c r="C1394" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1394" s="3" t="n">
@@ -64607,12 +64605,12 @@
       </c>
       <c r="B1395" s="2" t="inlineStr">
         <is>
-          <t>SET NIÑA CAUCHOS CAIMENES COLEROS</t>
+          <t>SET NIÃ‘A CAUCHOS CAIMENES COLEROS</t>
         </is>
       </c>
       <c r="C1395" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1395" s="3" t="n">
@@ -64653,12 +64651,12 @@
       </c>
       <c r="B1396" s="2" t="inlineStr">
         <is>
-          <t>BOLSA LIBRO DE AGUA PEQUEÑO 19CM X 15CM</t>
+          <t>BOLSA LIBRO DE AGUA PEQUEÃ‘O 19CM X 15CM</t>
         </is>
       </c>
       <c r="C1396" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1396" s="3" t="n">
@@ -64704,7 +64702,7 @@
       </c>
       <c r="C1397" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1397" s="3" t="n">
@@ -64750,7 +64748,7 @@
       </c>
       <c r="C1398" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1398" s="3" t="n">
@@ -64796,7 +64794,7 @@
       </c>
       <c r="C1399" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1399" s="3" t="n">
@@ -64842,7 +64840,7 @@
       </c>
       <c r="C1400" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1400" s="3" t="n">
@@ -64888,7 +64886,7 @@
       </c>
       <c r="C1401" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1401" s="3" t="n">
@@ -64934,7 +64932,7 @@
       </c>
       <c r="C1402" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1402" s="3" t="n">
@@ -64980,7 +64978,7 @@
       </c>
       <c r="C1403" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1403" s="3" t="n">
@@ -65026,7 +65024,7 @@
       </c>
       <c r="C1404" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1404" s="3" t="n">
@@ -65067,12 +65065,12 @@
       </c>
       <c r="B1405" s="2" t="inlineStr">
         <is>
-          <t>CAJA KIT DE UÑAS</t>
+          <t>CAJA KIT DE UÃ‘AS</t>
         </is>
       </c>
       <c r="C1405" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1405" s="3" t="n">
@@ -65113,12 +65111,12 @@
       </c>
       <c r="B1406" s="2" t="inlineStr">
         <is>
-          <t>SET ANILLOS NIÑA X12 KITTY CORAZON</t>
+          <t>SET ANILLOS NIÃ‘A X12 KITTY CORAZON</t>
         </is>
       </c>
       <c r="C1406" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1406" s="3" t="n">
@@ -65164,7 +65162,7 @@
       </c>
       <c r="C1407" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1407" s="3" t="n">
@@ -65210,7 +65208,7 @@
       </c>
       <c r="C1408" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1408" s="3" t="n">
@@ -65256,7 +65254,7 @@
       </c>
       <c r="C1409" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1409" s="3" t="n">
@@ -65302,7 +65300,7 @@
       </c>
       <c r="C1410" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1410" s="3" t="n">
@@ -65348,7 +65346,7 @@
       </c>
       <c r="C1411" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1411" s="3" t="n">
@@ -65394,7 +65392,7 @@
       </c>
       <c r="C1412" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1412" s="3" t="n">
@@ -65440,7 +65438,7 @@
       </c>
       <c r="C1413" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1413" s="3" t="n">
@@ -65486,7 +65484,7 @@
       </c>
       <c r="C1414" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1414" s="3" t="n">
@@ -65532,7 +65530,7 @@
       </c>
       <c r="C1415" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1415" s="3" t="n">
@@ -65578,7 +65576,7 @@
       </c>
       <c r="C1416" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1416" s="3" t="n">
@@ -65624,7 +65622,7 @@
       </c>
       <c r="C1417" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1417" s="3" t="n">
@@ -65670,7 +65668,7 @@
       </c>
       <c r="C1418" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1418" s="3" t="n">
@@ -65716,7 +65714,7 @@
       </c>
       <c r="C1419" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1419" s="3" t="n">
@@ -65762,7 +65760,7 @@
       </c>
       <c r="C1420" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1420" s="3" t="n">
@@ -65808,7 +65806,7 @@
       </c>
       <c r="C1421" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1421" s="3" t="n">
@@ -65854,7 +65852,7 @@
       </c>
       <c r="C1422" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1422" s="3" t="n">
@@ -65900,7 +65898,7 @@
       </c>
       <c r="C1423" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1423" s="3" t="n">
@@ -65946,7 +65944,7 @@
       </c>
       <c r="C1424" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1424" s="3" t="n">
@@ -65992,7 +65990,7 @@
       </c>
       <c r="C1425" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1425" s="3" t="n">
@@ -66038,7 +66036,7 @@
       </c>
       <c r="C1426" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1426" s="3" t="n">
@@ -66084,7 +66082,7 @@
       </c>
       <c r="C1427" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1427" s="3" t="n">
@@ -66130,7 +66128,7 @@
       </c>
       <c r="C1428" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1428" s="3" t="n">
@@ -66176,7 +66174,7 @@
       </c>
       <c r="C1429" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1429" s="3" t="n">
@@ -66222,7 +66220,7 @@
       </c>
       <c r="C1430" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1430" s="3" t="n">
@@ -66268,7 +66266,7 @@
       </c>
       <c r="C1431" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1431" s="3" t="n">
@@ -66314,7 +66312,7 @@
       </c>
       <c r="C1432" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1432" s="3" t="n">
@@ -66360,7 +66358,7 @@
       </c>
       <c r="C1433" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1433" s="3" t="n">
@@ -66406,7 +66404,7 @@
       </c>
       <c r="C1434" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1434" s="3" t="n">
@@ -66452,7 +66450,7 @@
       </c>
       <c r="C1435" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1435" s="3" t="n">
@@ -66498,7 +66496,7 @@
       </c>
       <c r="C1436" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1436" s="3" t="n">
@@ -66544,7 +66542,7 @@
       </c>
       <c r="C1437" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1437" s="3" t="n">
@@ -66590,7 +66588,7 @@
       </c>
       <c r="C1438" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1438" s="3" t="n">
@@ -66631,12 +66629,12 @@
       </c>
       <c r="B1439" s="2" t="inlineStr">
         <is>
-          <t>MUÑECA CON ACCESORIOS</t>
+          <t>MUÃ‘ECA CON ACCESORIOS</t>
         </is>
       </c>
       <c r="C1439" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1439" s="3" t="n">
@@ -66682,7 +66680,7 @@
       </c>
       <c r="C1440" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1440" s="3" t="n">
@@ -66728,7 +66726,7 @@
       </c>
       <c r="C1441" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1441" s="3" t="n">
@@ -66774,7 +66772,7 @@
       </c>
       <c r="C1442" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1442" s="3" t="n">
@@ -66820,7 +66818,7 @@
       </c>
       <c r="C1443" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1443" s="3" t="n">
@@ -66866,7 +66864,7 @@
       </c>
       <c r="C1444" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1444" s="3" t="n">
@@ -66912,7 +66910,7 @@
       </c>
       <c r="C1445" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1445" s="3" t="n">
@@ -66958,7 +66956,7 @@
       </c>
       <c r="C1446" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1446" s="3" t="n">
@@ -67004,7 +67002,7 @@
       </c>
       <c r="C1447" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1447" s="3" t="n">
@@ -67050,7 +67048,7 @@
       </c>
       <c r="C1448" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1448" s="3" t="n">
@@ -67096,7 +67094,7 @@
       </c>
       <c r="C1449" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1449" s="3" t="n">
@@ -67142,7 +67140,7 @@
       </c>
       <c r="C1450" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1450" s="3" t="n">
@@ -67188,7 +67186,7 @@
       </c>
       <c r="C1451" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1451" s="3" t="n">
@@ -67234,7 +67232,7 @@
       </c>
       <c r="C1452" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1452" s="3" t="n">
@@ -67280,7 +67278,7 @@
       </c>
       <c r="C1453" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1453" s="3" t="n">
@@ -67326,7 +67324,7 @@
       </c>
       <c r="C1454" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1454" s="3" t="n">
@@ -67372,7 +67370,7 @@
       </c>
       <c r="C1455" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1455" s="3" t="n">
@@ -67418,7 +67416,7 @@
       </c>
       <c r="C1456" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1456" s="3" t="n">
@@ -67464,7 +67462,7 @@
       </c>
       <c r="C1457" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1457" s="3" t="n">
@@ -67510,7 +67508,7 @@
       </c>
       <c r="C1458" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1458" s="3" t="n">
@@ -67556,7 +67554,7 @@
       </c>
       <c r="C1459" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1459" s="3" t="n">
@@ -67602,7 +67600,7 @@
       </c>
       <c r="C1460" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1460" s="3" t="n">
@@ -67648,7 +67646,7 @@
       </c>
       <c r="C1461" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1461" s="3" t="n">
@@ -67694,7 +67692,7 @@
       </c>
       <c r="C1462" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1462" s="3" t="n">
@@ -67735,12 +67733,12 @@
       </c>
       <c r="B1463" s="2" t="inlineStr">
         <is>
-          <t>ALCANCIA DIDACTICA PEQUEÑA</t>
+          <t>ALCANCIA DIDACTICA PEQUEÃ‘A</t>
         </is>
       </c>
       <c r="C1463" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1463" s="3" t="n">
@@ -67786,7 +67784,7 @@
       </c>
       <c r="C1464" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1464" s="3" t="n">
@@ -67832,7 +67830,7 @@
       </c>
       <c r="C1465" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1465" s="3" t="n">
@@ -67878,7 +67876,7 @@
       </c>
       <c r="C1466" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1466" s="3" t="n">
@@ -67924,7 +67922,7 @@
       </c>
       <c r="C1467" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1467" s="3" t="n">
@@ -67970,7 +67968,7 @@
       </c>
       <c r="C1468" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1468" s="3" t="n">
@@ -68016,7 +68014,7 @@
       </c>
       <c r="C1469" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1469" s="3" t="n">
@@ -68062,7 +68060,7 @@
       </c>
       <c r="C1470" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1470" s="3" t="n">
@@ -68108,7 +68106,7 @@
       </c>
       <c r="C1471" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1471" s="3" t="n">
@@ -68154,7 +68152,7 @@
       </c>
       <c r="C1472" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1472" s="3" t="n">
@@ -68200,7 +68198,7 @@
       </c>
       <c r="C1473" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1473" s="3" t="n">
@@ -68241,12 +68239,12 @@
       </c>
       <c r="B1474" s="2" t="inlineStr">
         <is>
-          <t>BOLSA SAPO SALTARINA DE JUGUETE PEQUEÑO</t>
+          <t>BOLSA SAPO SALTARINA DE JUGUETE PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1474" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1474" s="3" t="n">
@@ -68292,7 +68290,7 @@
       </c>
       <c r="C1475" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1475" s="3" t="n">
@@ -68338,7 +68336,7 @@
       </c>
       <c r="C1476" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1476" s="3" t="n">
@@ -68384,7 +68382,7 @@
       </c>
       <c r="C1477" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1477" s="3" t="n">
@@ -68430,7 +68428,7 @@
       </c>
       <c r="C1478" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1478" s="3" t="n">
@@ -68476,7 +68474,7 @@
       </c>
       <c r="C1479" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1479" s="3" t="n">
@@ -68517,12 +68515,12 @@
       </c>
       <c r="B1480" s="2" t="inlineStr">
         <is>
-          <t>PELOTA ANTIESTRÉS 9 MOTIVOS (DK3019-2-3-7-5-9-12-13)DK284</t>
+          <t>PELOTA ANTIESTRÃ‰S 9 MOTIVOS (DK3019-2-3-7-5-9-12-13)DK284</t>
         </is>
       </c>
       <c r="C1480" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1480" s="3" t="n">
@@ -68568,7 +68566,7 @@
       </c>
       <c r="C1481" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1481" s="3" t="n">
@@ -68614,7 +68612,7 @@
       </c>
       <c r="C1482" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1482" s="3" t="n">
@@ -68660,7 +68658,7 @@
       </c>
       <c r="C1483" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1483" s="3" t="n">
@@ -68706,7 +68704,7 @@
       </c>
       <c r="C1484" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1484" s="3" t="n">
@@ -68752,7 +68750,7 @@
       </c>
       <c r="C1485" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1485" s="3" t="n">
@@ -68798,7 +68796,7 @@
       </c>
       <c r="C1486" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1486" s="3" t="n">
@@ -68844,7 +68842,7 @@
       </c>
       <c r="C1487" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1487" s="3" t="n">
@@ -68890,7 +68888,7 @@
       </c>
       <c r="C1488" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1488" s="3" t="n">
@@ -68936,7 +68934,7 @@
       </c>
       <c r="C1489" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1489" s="3" t="n">
@@ -68982,7 +68980,7 @@
       </c>
       <c r="C1490" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1490" s="3" t="n">
@@ -69028,7 +69026,7 @@
       </c>
       <c r="C1491" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1491" s="3" t="n">
@@ -69069,12 +69067,12 @@
       </c>
       <c r="B1492" s="2" t="inlineStr">
         <is>
-          <t>BOLSA JAZZ FICHA PEQUEÑA X200</t>
+          <t>BOLSA JAZZ FICHA PEQUEÃ‘A X200</t>
         </is>
       </c>
       <c r="C1492" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1492" s="3" t="n">
@@ -69120,7 +69118,7 @@
       </c>
       <c r="C1493" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1493" s="3" t="n">
@@ -69166,7 +69164,7 @@
       </c>
       <c r="C1494" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1494" s="3" t="n">
@@ -69207,12 +69205,12 @@
       </c>
       <c r="B1495" s="2" t="inlineStr">
         <is>
-          <t>BOLSA CARRO PIÑATERO</t>
+          <t>BOLSA CARRO PIÃ‘ATERO</t>
         </is>
       </c>
       <c r="C1495" s="2" t="inlineStr">
         <is>
-          <t>Piñatería</t>
+          <t>piÃ±ateria</t>
         </is>
       </c>
       <c r="D1495" s="3" t="n">
@@ -71599,7 +71597,7 @@
       </c>
       <c r="B1547" s="2" t="inlineStr">
         <is>
-          <t>SCUICHI LABUBU PEQUEÑA</t>
+          <t>SCUICHI LABUBU PEQUEÃ‘A</t>
         </is>
       </c>
       <c r="C1547" s="2" t="inlineStr">
@@ -71645,7 +71643,7 @@
       </c>
       <c r="B1548" s="2" t="inlineStr">
         <is>
-          <t>SCUICHI CAPIBARA PEQUEÑO</t>
+          <t>SCUICHI CAPIBARA PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1548" s="2" t="inlineStr">
@@ -72197,7 +72195,7 @@
       </c>
       <c r="B1560" s="2" t="inlineStr">
         <is>
-          <t>SLIME KURUMI TARRO PEQUEÑO</t>
+          <t>SLIME KURUMI TARRO PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1560" s="2" t="inlineStr">
@@ -72427,7 +72425,7 @@
       </c>
       <c r="B1565" s="2" t="inlineStr">
         <is>
-          <t>SLIME OSO TARRO PEQUEÑO</t>
+          <t>SLIME OSO TARRO PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1565" s="2" t="inlineStr">
@@ -72841,7 +72839,7 @@
       </c>
       <c r="B1574" s="2" t="inlineStr">
         <is>
-          <t>SLIME LEON PEQUEÑO</t>
+          <t>SLIME LEON PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1574" s="2" t="inlineStr">
@@ -72887,7 +72885,7 @@
       </c>
       <c r="B1575" s="2" t="inlineStr">
         <is>
-          <t>SLIME MARIQUITA PEQUEÑO</t>
+          <t>SLIME MARIQUITA PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1575" s="2" t="inlineStr">
@@ -72933,7 +72931,7 @@
       </c>
       <c r="B1576" s="2" t="inlineStr">
         <is>
-          <t>SLIME TORTUGA PEQUEÑO</t>
+          <t>SLIME TORTUGA PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1576" s="2" t="inlineStr">
@@ -72979,7 +72977,7 @@
       </c>
       <c r="B1577" s="2" t="inlineStr">
         <is>
-          <t>SLIME PATO PEQUEÑO</t>
+          <t>SLIME PATO PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1577" s="2" t="inlineStr">
@@ -73025,7 +73023,7 @@
       </c>
       <c r="B1578" s="2" t="inlineStr">
         <is>
-          <t>SLIME PERRO PEQUEÑO</t>
+          <t>SLIME PERRO PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1578" s="2" t="inlineStr">
@@ -73071,7 +73069,7 @@
       </c>
       <c r="B1579" s="2" t="inlineStr">
         <is>
-          <t>SLIME OSO I LOVE YOU PEQUEÑO</t>
+          <t>SLIME OSO I LOVE YOU PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1579" s="2" t="inlineStr">
@@ -73117,7 +73115,7 @@
       </c>
       <c r="B1580" s="2" t="inlineStr">
         <is>
-          <t>SLIME HIPOPOTAMO PEQUEÑO</t>
+          <t>SLIME HIPOPOTAMO PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1580" s="2" t="inlineStr">
@@ -73163,7 +73161,7 @@
       </c>
       <c r="B1581" s="2" t="inlineStr">
         <is>
-          <t>SLIME PANAL PEQUEÑO</t>
+          <t>SLIME PANAL PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1581" s="2" t="inlineStr">
@@ -73209,7 +73207,7 @@
       </c>
       <c r="B1582" s="2" t="inlineStr">
         <is>
-          <t>SLIME PULPO PEQUEÑO</t>
+          <t>SLIME PULPO PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1582" s="2" t="inlineStr">
@@ -73255,7 +73253,7 @@
       </c>
       <c r="B1583" s="2" t="inlineStr">
         <is>
-          <t>SLIME GATO PEQUEÑO</t>
+          <t>SLIME GATO PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1583" s="2" t="inlineStr">
@@ -73301,7 +73299,7 @@
       </c>
       <c r="B1584" s="2" t="inlineStr">
         <is>
-          <t>SLIME OSO GAFAS PEQUEÑO</t>
+          <t>SLIME OSO GAFAS PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1584" s="2" t="inlineStr">
@@ -73347,7 +73345,7 @@
       </c>
       <c r="B1585" s="2" t="inlineStr">
         <is>
-          <t>SLIME HELLO KITY PEQUEÑO</t>
+          <t>SLIME HELLO KITY PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1585" s="2" t="inlineStr">
@@ -73393,7 +73391,7 @@
       </c>
       <c r="B1586" s="2" t="inlineStr">
         <is>
-          <t>SLIME OREJAS PEQUEÑO</t>
+          <t>SLIME OREJAS PEQUEÃ‘O</t>
         </is>
       </c>
       <c r="C1586" s="2" t="inlineStr">
@@ -73945,7 +73943,7 @@
       </c>
       <c r="B1598" s="2" t="inlineStr">
         <is>
-          <t>TERMO DISEÑO SURTIDO GRANDE</t>
+          <t>TERMO DISEÃ‘O SURTIDO GRANDE</t>
         </is>
       </c>
       <c r="C1598" s="2" t="inlineStr">
@@ -74175,7 +74173,7 @@
       </c>
       <c r="B1603" s="2" t="inlineStr">
         <is>
-          <t>TERMO DISEÑO SURTIDO 4 COLORES</t>
+          <t>TERMO DISEÃ‘O SURTIDO 4 COLORES</t>
         </is>
       </c>
       <c r="C1603" s="2" t="inlineStr">
@@ -74221,7 +74219,7 @@
       </c>
       <c r="B1604" s="2" t="inlineStr">
         <is>
-          <t>TERMO DISEÑO SURTIDO 4 MODELOS</t>
+          <t>TERMO DISEÃ‘O SURTIDO 4 MODELOS</t>
         </is>
       </c>
       <c r="C1604" s="2" t="inlineStr">
@@ -74267,7 +74265,7 @@
       </c>
       <c r="B1605" s="2" t="inlineStr">
         <is>
-          <t>TERMO DISEÑOS SURTIDOS 4 COLORES</t>
+          <t>TERMO DISEÃ‘OS SURTIDOS 4 COLORES</t>
         </is>
       </c>
       <c r="C1605" s="2" t="inlineStr">
@@ -74313,7 +74311,7 @@
       </c>
       <c r="B1606" s="2" t="inlineStr">
         <is>
-          <t>TERMO DISEÑOS SURTIDOS 3 COLORES</t>
+          <t>TERMO DISEÃ‘OS SURTIDOS 3 COLORES</t>
         </is>
       </c>
       <c r="C1606" s="2" t="inlineStr">
@@ -74359,7 +74357,7 @@
       </c>
       <c r="B1607" s="2" t="inlineStr">
         <is>
-          <t>TERMO DISEÑO SURTIDO 4 COLORES</t>
+          <t>TERMO DISEÃ‘O SURTIDO 4 COLORES</t>
         </is>
       </c>
       <c r="C1607" s="2" t="inlineStr">
@@ -74497,7 +74495,7 @@
       </c>
       <c r="B1610" s="2" t="inlineStr">
         <is>
-          <t>TERMO DISEÑO SURTIDO 4 COLORES</t>
+          <t>TERMO DISEÃ‘O SURTIDO 4 COLORES</t>
         </is>
       </c>
       <c r="C1610" s="2" t="inlineStr">
@@ -74589,7 +74587,7 @@
       </c>
       <c r="B1612" s="2" t="inlineStr">
         <is>
-          <t>TERMO DISEÑO SURTIDO 5 COLORES</t>
+          <t>TERMO DISEÃ‘O SURTIDO 5 COLORES</t>
         </is>
       </c>
       <c r="C1612" s="2" t="inlineStr">
@@ -75377,78 +75375,78 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-12 20:40</t>
+          <t>2026-10-12 22:46</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Productos en Juguetería</t>
+          <t>Productos en Animales</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>287</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Productos en Piñatería</t>
+          <t>Productos en Armatodo</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>259</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Productos en Juego de mesa</t>
+          <t>Productos en Bebé</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>206</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Productos en Armatodo</t>
+          <t>Productos en Burbujeros</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>170</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Productos en Didáctico</t>
+          <t>Productos en Cacharro</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>163</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Productos en Slime</t>
+          <t>Productos en Colecciones</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>98</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Productos en Cacharro</t>
+          <t>Productos en Cubo Rubik</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>80</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -75464,91 +75462,91 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Productos en Peluches</t>
+          <t>Productos en Didáctico</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>61</v>
+        <v>163</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Productos en Colecciones</t>
+          <t>Productos en Escolar</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>47</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Productos en Bebé</t>
+          <t>Productos en Hogar</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Productos en Termos</t>
+          <t>Productos en Juego de mesa</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>34</v>
+        <v>206</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Productos en Burbujeros</t>
+          <t>Productos en Juguetería</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>31</v>
+        <v>287</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Productos en Escolar</t>
+          <t>Productos en Peluches</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>27</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Productos en Animales</t>
+          <t>Productos en piÃ±ateria</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>26</v>
+        <v>259</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Productos en Cubo Rubik</t>
+          <t>Productos en Slime</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>18</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Productos en Hogar</t>
+          <t>Productos en Termos</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>